<commit_message>
Add T4 to tests.
Add t4
</commit_message>
<xml_diff>
--- a/Reference/Mitigations Tests.xlsx
+++ b/Reference/Mitigations Tests.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\GitHub\tdm-ghg-calculator\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{177BCFCA-631C-44C8-B3E6-77478DE56CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACDF4679-B3B3-4200-8643-A758A0FE23BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T1" sheetId="1" r:id="rId1"/>
     <sheet name="T2" sheetId="2" r:id="rId2"/>
     <sheet name="T3" sheetId="3" r:id="rId3"/>
+    <sheet name="T4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="4">
   <si>
     <t>B</t>
   </si>
@@ -461,7 +462,7 @@
         <v>0</v>
       </c>
       <c r="B1">
-        <v>4</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -477,7 +478,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>90</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -485,8 +486,43 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <f>(B2*B1)/-B3</f>
+        <f>-(B2*B1)/B3</f>
         <v>-0.21777777777777779</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D486991-6FF1-4805-9025-F98917C073B8}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>-0.28599999999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <f>B2*B1</f>
+        <v>-5.7200000000000001E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update sheet for tests.
Update sheet
</commit_message>
<xml_diff>
--- a/Reference/Mitigations Tests.xlsx
+++ b/Reference/Mitigations Tests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\GitHub\tdm-ghg-calculator\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{760DE46B-1A41-4CB7-AC98-FEEFDD21227B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B86DC95-EB8D-4FC3-B7BC-412313083EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,11 @@
     <sheet name="T4" sheetId="4" r:id="rId4"/>
     <sheet name="T55" sheetId="5" r:id="rId5"/>
     <sheet name="T5" sheetId="6" r:id="rId6"/>
+    <sheet name="T6" sheetId="7" r:id="rId7"/>
+    <sheet name="T7" sheetId="8" r:id="rId8"/>
+    <sheet name="T8" sheetId="9" r:id="rId9"/>
+    <sheet name="T9" sheetId="10" r:id="rId10"/>
+    <sheet name="T11" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="9">
   <si>
     <t>B</t>
   </si>
@@ -53,6 +58,21 @@
   </si>
   <si>
     <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>I</t>
   </si>
 </sst>
 </file>
@@ -88,8 +108,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -411,6 +432,158 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B16458-C940-4002-A635-0E8C338DCCC2}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>-0.43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <f>(B2/B1)*B3*B4*B5*B6*B7*B8</f>
+        <v>-2.6144000000000004E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8198844C-4C52-40D3-A5CC-C3F133397CB1}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>2.7E-2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>307.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>763.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <f>((1-B1)*B2*B5+B1*(B3/B4)*B6)/((1-B1)*B2*B5+B1*B3*B5) -1</f>
+        <v>-3.3192034620550204E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A31D2A21-89B6-449E-AB74-EE9FEB6BE116}">
   <dimension ref="A1:B4"/>
@@ -609,4 +782,128 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D512145F-AAB1-4862-93C2-E8C630C31BD4}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>-0.26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <f>B1*B2*B3</f>
+        <v>-0.221</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BE34028-78B5-4730-BB77-EDE25BEED080}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <f>B1*B2*B3</f>
+        <v>-2.7999999999999997E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6836B869-383D-4226-9FF3-A319F5FB364A}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <f>0.08</f>
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <f>B1*B2</f>
+        <v>4.8000000000000001E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
T 22 C + D Tests
Scooter and transition to electric bike share tests.
</commit_message>
<xml_diff>
--- a/Reference/Mitigations Tests.xlsx
+++ b/Reference/Mitigations Tests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\GitHub\tdm-ghg-calculator\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1813BF93-D1F8-4E46-AEF9-A7BE0F4CAE6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70B8738-5839-4B1A-AB24-6DE943C2D0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="13770" firstSheet="18" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="13770" firstSheet="21" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T1" sheetId="1" r:id="rId1"/>
@@ -35,13 +35,16 @@
     <sheet name="T20" sheetId="28" r:id="rId20"/>
     <sheet name="T21a" sheetId="19" r:id="rId21"/>
     <sheet name="T22a" sheetId="29" r:id="rId22"/>
-    <sheet name="T21b" sheetId="20" r:id="rId23"/>
-    <sheet name="T22cB" sheetId="21" r:id="rId24"/>
-    <sheet name="T23" sheetId="22" r:id="rId25"/>
-    <sheet name="T24B" sheetId="23" r:id="rId26"/>
-    <sheet name="T25B" sheetId="24" r:id="rId27"/>
-    <sheet name="T26" sheetId="25" r:id="rId28"/>
-    <sheet name="T27" sheetId="27" r:id="rId29"/>
+    <sheet name="T22b" sheetId="30" r:id="rId23"/>
+    <sheet name="T22c" sheetId="32" r:id="rId24"/>
+    <sheet name="T22d" sheetId="31" r:id="rId25"/>
+    <sheet name="T21b" sheetId="20" r:id="rId26"/>
+    <sheet name="T22cB" sheetId="21" r:id="rId27"/>
+    <sheet name="T23" sheetId="22" r:id="rId28"/>
+    <sheet name="T24B" sheetId="23" r:id="rId29"/>
+    <sheet name="T25B" sheetId="24" r:id="rId30"/>
+    <sheet name="T26" sheetId="25" r:id="rId31"/>
+    <sheet name="T27" sheetId="27" r:id="rId32"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="12">
   <si>
     <t>B</t>
   </si>
@@ -106,6 +109,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -141,13 +147,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1337,6 +1344,249 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFB0BC64-71B3-4F79-95ED-EE6427AF4050}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>9.7200000000000006</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8">
+        <f>(((B2-B1)*B3*B4*B5)/(B6*B7))*-1</f>
+        <v>-3.3327617741197988E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{953B5401-36F7-4AFE-839C-026FA056AD0B}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.38500000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>2.14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>9.7200000000000006</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8">
+        <f>(((B2-B1)*B3*B4*B5)/(B6*B7))*-1</f>
+        <v>-5.6038008687700046E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{027E8AEE-0803-4B02-9E46-BDF34BF75B33}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>0.19600000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>9.6999999999999993</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="4">
+        <f>(((-B1*B2*B3*((B4*B5)-(B6*B7)))/(B8*B9)))</f>
+        <v>-4.2379948453608247E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8988892F-DED0-46F4-AA2C-CCF2CC1ADF7C}">
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1431,7 +1681,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CD9EE00-52A7-487E-921D-B9FCCC55DCBC}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1507,7 +1757,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0D036EF-8CF1-4C13-9B46-8108C0132C37}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1566,7 +1816,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{105B05B6-310E-40FF-A289-A462CFD2CD1A}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1642,7 +1892,50 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56180196-4A51-42CE-9237-42DECB8F409D}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>4.9000000000000004</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <f>-(B2*B1)/B3</f>
+        <v>-0.21777777777777779</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5EE5C2E-1F2E-408A-BC54-0F14E725BF63}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1709,7 +2002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF5EF6D2-2159-4E97-8BF0-19BB3D566A71}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1776,7 +2069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4E4C011-9C8B-4490-8B6D-F742F24FB084}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1843,49 +2136,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56180196-4A51-42CE-9237-42DECB8F409D}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>4.9000000000000004</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4">
-        <f>-(B2*B1)/B3</f>
-        <v>-0.21777777777777779</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D486991-6FF1-4805-9025-F98917C073B8}">
   <dimension ref="A1:B3"/>

</xml_diff>

<commit_message>
T29 Test + T22B Fix
Try to fix T22B test and add T29 reduce fares.
</commit_message>
<xml_diff>
--- a/Reference/Mitigations Tests.xlsx
+++ b/Reference/Mitigations Tests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\GitHub\tdm-ghg-calculator\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D89637-0070-4658-A0F4-803531A458F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3BC9283-0E6C-4BCE-8C3E-6938DB103540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="13770" firstSheet="23" activeTab="32" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="13770" firstSheet="28" activeTab="33" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T1" sheetId="1" r:id="rId1"/>
@@ -46,6 +46,7 @@
     <sheet name="T26" sheetId="25" r:id="rId31"/>
     <sheet name="T27" sheetId="27" r:id="rId32"/>
     <sheet name="T28" sheetId="33" r:id="rId33"/>
+    <sheet name="T29B" sheetId="34" r:id="rId34"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -68,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="12">
   <si>
     <t>B</t>
   </si>
@@ -1386,7 +1387,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -1411,7 +1412,7 @@
       </c>
       <c r="B8">
         <f>(((B2-B1)*B3*B4*B5)/(B6*B7))*-1</f>
-        <v>-3.3327617741197988E-4</v>
+        <v>-4.9991426611796985E-4</v>
       </c>
     </row>
   </sheetData>
@@ -2229,6 +2230,74 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24D4371F-7752-4380-AAD2-3CD65C64C4E4}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0.57799999999999996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <f>(B1*B2*B3*B4*B6)/B5</f>
+        <v>-1.0403999999999998E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D486991-6FF1-4805-9025-F98917C073B8}">
   <dimension ref="A1:B3"/>

</xml_diff>

<commit_message>
Add T40 + T56 Tests
Tests for school programs.
</commit_message>
<xml_diff>
--- a/Reference/Mitigations Tests.xlsx
+++ b/Reference/Mitigations Tests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\GitHub\tdm-ghg-calculator\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C99B3DB-3519-42D1-B6CA-2FD5E6829C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C0D2785-4AD4-4B40-ADC3-8972F8C463F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="13770" firstSheet="28" activeTab="34" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="13770" firstSheet="31" activeTab="36" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,9 @@
     <sheet name="T27" sheetId="27" r:id="rId32"/>
     <sheet name="T28" sheetId="33" r:id="rId33"/>
     <sheet name="T29B" sheetId="34" r:id="rId34"/>
-    <sheet name="T46" sheetId="35" r:id="rId35"/>
+    <sheet name="T40" sheetId="36" r:id="rId35"/>
+    <sheet name="T46" sheetId="35" r:id="rId36"/>
+    <sheet name="T56" sheetId="37" r:id="rId37"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -70,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="12">
   <si>
     <t>B</t>
   </si>
@@ -2300,32 +2302,32 @@
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E1BA039-FAE9-4F58-A255-BAD81FF0BAAA}">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>12000</v>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A9A9924-ECD5-42C9-AEB6-442F006B5576}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>0.79</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2333,7 +2335,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.15</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2341,7 +2343,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>0.83299999999999996</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2349,7 +2351,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>1.45</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2357,7 +2359,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.249</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -2365,6 +2367,90 @@
         <v>8</v>
       </c>
       <c r="B8">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <f>(B1*B2*B3*((B7/B4)-((B6*B8)/B5)))/(B7/B4)</f>
+        <v>-0.13844472023010548</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E1BA039-FAE9-4F58-A255-BAD81FF0BAAA}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>0.83299999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>0.249</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
         <v>0.20300000000000001</v>
       </c>
     </row>
@@ -2391,6 +2477,73 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83802985-441C-4BBF-B305-3743B0992738}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>8.66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <f>B2*B5*((B1-B3)/((B6*B4*(1-B2))+(B2*B3*B5)))</f>
+        <v>-2.6530420122039929E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D486991-6FF1-4805-9025-F98917C073B8}">
   <dimension ref="A1:B3"/>

</xml_diff>